<commit_message>
S27 - load-test dictionaries, equipment classes and registry entries
Six new codelist dictionaries for StaticLoadTest/RapidLoadTest/
DynamicLoadTest/LoadTestIncrement (loadingProcedure, testCategory,
analysisMethod, testMethod, referenceSystem, loadingPhase), each
researched against both ASTM and EN ISO 22477 terminology so the
vocabulary itself carries more than one governing standard rather than
assuming ASTM alone. properties.xml gains critical_creep_load,
closing Post-installation row 12. equipmentClass.xml gains
rapid_load_device and dynamic_test_hammer, completing the equipment
side alongside the already-present load_test_reaction_frame/
hydraulic_jack. The specification registry gains EN ISO 22477-1/-10/-4,
the direct European counterparts of the already-registered ASTM
D1143/D7383/D4945, so a StaticLoadTest/RapidLoadTest/DynamicLoadTest
can cite whichever standard(s) actually governed it.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/equipmentClass.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/equipmentClass.xlsx
@@ -1754,27 +1754,67 @@
     </row>
     <row r="31">
       <c r="A31" s="2">
-        <f>IF(ISNA(VLOOKUP(B31,AssociatedElements!B$2:B2969,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="B31" s="13" t="n"/>
-      <c r="C31" s="18" t="n"/>
-      <c r="D31" s="19" t="n"/>
-      <c r="E31" s="18" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B31,AssociatedElements!B$2:B$999,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>rapid_load_device</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="inlineStr">
+        <is>
+          <t>Rapid Load Test Device</t>
+        </is>
+      </c>
+      <c r="D31" s="19" t="inlineStr">
+        <is>
+          <t>The pneumatic or hydraulic force-pulse generator used to apply the load in a rapid load test - a Statnamic device or an equivalent force-pulse actuator, per ASTM D7383 or EN ISO 22477-10.</t>
+        </is>
+      </c>
+      <c r="E31" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F31" s="18" t="n"/>
-      <c r="G31" s="9" t="n"/>
+      <c r="G31" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2">
-        <f>IF(ISNA(VLOOKUP(B32,AssociatedElements!B$2:B2970,1,FALSE)),"Not used","")</f>
-        <v/>
-      </c>
-      <c r="B32" s="13" t="n"/>
-      <c r="C32" s="18" t="n"/>
-      <c r="D32" s="19" t="n"/>
-      <c r="E32" s="18" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B32,AssociatedElements!B$2:B$999,1,FALSE)),"Not used","")</f>
+        <v/>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>dynamic_test_hammer</t>
+        </is>
+      </c>
+      <c r="C32" s="18" t="inlineStr">
+        <is>
+          <t>Dynamic Load Test Hammer</t>
+        </is>
+      </c>
+      <c r="D32" s="19" t="inlineStr">
+        <is>
+          <t>The impact hammer used to apply the blow(s) in a high-strain dynamic load test, per ASTM D4945 or EN ISO 22477-4.</t>
+        </is>
+      </c>
+      <c r="E32" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F32" s="18" t="n"/>
-      <c r="G32" s="9" t="n"/>
+      <c r="G32" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2">
@@ -2343,17 +2383,35 @@
     </row>
     <row r="31">
       <c r="A31">
-        <f>IF(ISNA(VLOOKUP(B31,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B31" s="13" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B31,Definitions!B$2:B$999,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B31" s="13" t="inlineStr">
+        <is>
+          <t>rapid_load_device</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>//diggs:Equipment/diggs:class</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32">
-        <f>IF(ISNA(VLOOKUP(B32,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
-        <v/>
-      </c>
-      <c r="B32" s="13" t="n"/>
+        <f>IF(ISNA(VLOOKUP(B32,Definitions!B$2:B$999,1,FALSE)),"Not listed","")</f>
+        <v/>
+      </c>
+      <c r="B32" s="13" t="inlineStr">
+        <is>
+          <t>dynamic_test_hammer</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>//diggs:Equipment/diggs:class</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33">

</xml_diff>

<commit_message>
S29 - low-strain integrity test dictionaries, equipment class, and registry
New lowStrainTestMethod.xml (pulse_echo / transient_response), new
equipmentClass.xml#low_strain_impact_hammer, new properties.xml#defect_depth
(the low-strain integrity test's interpreted result). Registers NF P94-160-2
and NF P94-160-4, the French national counterparts to ASTM D5882's two
internal methods. Also flags the pre-existing astm_d5882 registry entry as
registryStatus=withdrawn (withdrawn by ASTM in 2025, no replacement named) -
a factual correction found while researching the standard, not previously
recorded.
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/equipmentClass.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/equipmentClass.xlsx
@@ -1821,12 +1821,32 @@
         <f>IF(ISNA(VLOOKUP(B33,AssociatedElements!B$2:B2971,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B33" s="13" t="n"/>
-      <c r="C33" s="18" t="n"/>
-      <c r="D33" s="19" t="n"/>
-      <c r="E33" s="18" t="n"/>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>low_strain_impact_hammer</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="inlineStr">
+        <is>
+          <t>Low-Strain Impact Hammer</t>
+        </is>
+      </c>
+      <c r="D33" s="19" t="inlineStr">
+        <is>
+          <t>The small handheld hammer (typically plastic- or rubber-tipped) used to apply the impact in a low-strain integrity test, per ASTM D5882 or NF P94-160-2/-4. Distinct from equipmentClass.xml#dynamic_test_hammer, the much larger drop or diesel hammer used to apply a high-strain blow in ASTM D4945 dynamic load testing - the two tests use different equipment at entirely different energy scales.</t>
+        </is>
+      </c>
+      <c r="E33" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F33" s="18" t="n"/>
-      <c r="G33" s="9" t="n"/>
+      <c r="G33" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2">
@@ -2418,7 +2438,16 @@
         <f>IF(ISNA(VLOOKUP(B33,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B33" s="13" t="n"/>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>low_strain_impact_hammer</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>//diggs:Equipment/diggs:class</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34">

</xml_diff>

<commit_message>
S31 - thermal integrity profiling dictionaries, equipment, and registry
New thermalIntegrityProfilingMethod.xml (thermal_probe / embedded_thermal_sensor
/ embedded_fiber_optic, ASTM D7949's three methods per its 2025 reinstatement),
two new equipmentClass.xml entries, new properties.xml#effective_radius plus a
third Occurrence on the pre-existing #temperature entry, new
measurementKind.xml#thermal_integrity_profiling, and a new astm_d7949 registry
entry recording the standard's 2023 withdrawal / 2025 reinstatement and the
absence of any European or ISO counterpart.
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/equipmentClass.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/equipmentClass.xlsx
@@ -1853,24 +1853,64 @@
         <f>IF(ISNA(VLOOKUP(B34,AssociatedElements!B$2:B2972,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B34" s="13" t="n"/>
-      <c r="C34" s="18" t="n"/>
-      <c r="D34" s="19" t="n"/>
-      <c r="E34" s="18" t="n"/>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>thermal_integrity_probe</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="inlineStr">
+        <is>
+          <t>Thermal Integrity Profiling Probe</t>
+        </is>
+      </c>
+      <c r="D34" s="19" t="inlineStr">
+        <is>
+          <t>The probe lowered into access ducts to take temperature readings in ASTM D7949 Method A thermal integrity profiling. Distinct from equipmentClass.xml#thermistor, which is the embedded sensor Method B uses instead - the two methods use different equipment classes for the same underlying measurement.</t>
+        </is>
+      </c>
+      <c r="E34" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F34" s="18" t="n"/>
-      <c r="G34" s="9" t="n"/>
+      <c r="G34" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2">
         <f>IF(ISNA(VLOOKUP(B35,AssociatedElements!B$2:B2973,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B35" s="13" t="n"/>
-      <c r="C35" s="18" t="n"/>
-      <c r="D35" s="19" t="n"/>
-      <c r="E35" s="18" t="n"/>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>embedded_fiber_optic_cable</t>
+        </is>
+      </c>
+      <c r="C35" s="18" t="inlineStr">
+        <is>
+          <t>Embedded Fiber-Optic Cable</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t>The fiber-optic cable attached to the reinforcing cage and cast into the concrete for ASTM D7949 Method C thermal integrity profiling, giving effectively continuous temperature coverage along the element's length.</t>
+        </is>
+      </c>
+      <c r="E35" s="18" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F35" s="18" t="n"/>
-      <c r="G35" s="9" t="n"/>
+      <c r="G35" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2">
@@ -2454,14 +2494,32 @@
         <f>IF(ISNA(VLOOKUP(B34,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B34" s="13" t="n"/>
+      <c r="B34" s="13" t="inlineStr">
+        <is>
+          <t>thermal_integrity_probe</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>//diggs:Equipment/diggs:class</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35">
         <f>IF(ISNA(VLOOKUP(B35,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B35" s="13" t="n"/>
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>embedded_fiber_optic_cable</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>//diggs:Equipment/diggs:class</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36">

</xml_diff>